<commit_message>
updated readings of exp_7
</commit_message>
<xml_diff>
--- a/EXP_7/READINGS/Book1.xlsx
+++ b/EXP_7/READINGS/Book1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EDC_LAB\EXP_7\READINGS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18F00609-7763-4DC1-9654-0BB1F86EBA61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEF84BCA-0388-49D5-8C9F-B4F8B65314B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{65FFEAC9-52A6-42D7-AA78-72B4541954C9}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
   <si>
     <t>CURRENT MIRROR</t>
   </si>
@@ -45,9 +45,6 @@
     <t>VOUT</t>
   </si>
   <si>
-    <t>`</t>
-  </si>
-  <si>
     <t>V(X AXIS)</t>
   </si>
   <si>
@@ -84,13 +81,31 @@
     <t>47 ohm</t>
   </si>
   <si>
-    <t>iout</t>
-  </si>
-  <si>
-    <t>vbias = 3v</t>
-  </si>
-  <si>
-    <t>100 ohm</t>
+    <t>vbias =7v</t>
+  </si>
+  <si>
+    <t>188mv</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>190mv</t>
+  </si>
+  <si>
+    <t>56 ohm</t>
+  </si>
+  <si>
+    <t>82 ohm</t>
+  </si>
+  <si>
+    <t>192 mv</t>
+  </si>
+  <si>
+    <t>vin = 200mv</t>
+  </si>
+  <si>
+    <t>unloaded vout=192mv</t>
   </si>
 </sst>
 </file>
@@ -180,8 +195,13 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-IN"/>
-              <a:t>VIN &amp; VOUT</a:t>
+              <a:t>VIN</a:t>
             </a:r>
+            <a:r>
+              <a:rPr lang="en-IN" baseline="0"/>
+              <a:t> &amp; VOUT</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-IN"/>
           </a:p>
         </c:rich>
       </c:tx>
@@ -260,10 +280,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$5:$A$14</c:f>
+              <c:f>Sheet1!$A$5:$A$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
                   <c:v>1.5</c:v>
                 </c:pt>
@@ -290,19 +310,16 @@
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>9.5</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>10.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$B$5:$B$14</c:f>
+              <c:f>Sheet1!$B$5:$B$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
                   <c:v>1.5</c:v>
                 </c:pt>
@@ -329,9 +346,6 @@
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>9.5</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>10.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -339,7 +353,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-8568-4A35-A2DC-10024AB8460B}"/>
+              <c16:uniqueId val="{00000000-188B-4C97-8717-CE31039589EF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -383,10 +397,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$5:$A$14</c:f>
+              <c:f>Sheet1!$A$5:$A$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
                   <c:v>1.5</c:v>
                 </c:pt>
@@ -413,48 +427,42 @@
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>9.5</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>10.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$C$5:$C$14</c:f>
+              <c:f>Sheet1!$C$5:$C$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>2</c:v>
+                  <c:v>0.71</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.1</c:v>
+                  <c:v>1.7</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.0999999999999996</c:v>
+                  <c:v>2.69</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.9000000000000004</c:v>
+                  <c:v>3.67</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5.6</c:v>
+                  <c:v>4.66</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>6.3</c:v>
+                  <c:v>5.64</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6.7</c:v>
+                  <c:v>6.62</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7</c:v>
+                  <c:v>7.59</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7.6</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>8.4</c:v>
+                  <c:v>8.5299999999999994</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -462,7 +470,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-8568-4A35-A2DC-10024AB8460B}"/>
+              <c16:uniqueId val="{00000001-188B-4C97-8717-CE31039589EF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -474,11 +482,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="434719615"/>
-        <c:axId val="511336399"/>
+        <c:axId val="1856451071"/>
+        <c:axId val="1697871663"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="434719615"/>
+        <c:axId val="1856451071"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -535,12 +543,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="511336399"/>
+        <c:crossAx val="1697871663"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="511336399"/>
+        <c:axId val="1697871663"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -597,7 +605,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="434719615"/>
+        <c:crossAx val="1856451071"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1244,23 +1252,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>556260</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>102870</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>563880</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>251460</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>102870</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>259080</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
+        <xdr:cNvPr id="3" name="Chart 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{234C808F-6E3C-03F5-8524-996003CFC1A7}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ABC3F6EA-2FEA-7E84-841A-F296A20B5F49}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1578,22 +1586,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A02E8E98-0582-4189-8980-F13E4F53E866}">
-  <dimension ref="A2:F44"/>
+  <dimension ref="A2:C49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>1</v>
@@ -1602,7 +1610,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1.5</v>
       </c>
@@ -1610,10 +1618,10 @@
         <v>1.5</v>
       </c>
       <c r="C5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2.5</v>
       </c>
@@ -1621,10 +1629,10 @@
         <v>2.5</v>
       </c>
       <c r="C6">
-        <v>3.1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>3.5</v>
       </c>
@@ -1632,10 +1640,10 @@
         <v>3.5</v>
       </c>
       <c r="C7">
-        <v>4.0999999999999996</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+        <v>2.69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>4.5</v>
       </c>
@@ -1643,10 +1651,10 @@
         <v>4.5</v>
       </c>
       <c r="C8">
-        <v>4.9000000000000004</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+        <v>3.67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>5.5</v>
       </c>
@@ -1654,13 +1662,10 @@
         <v>5.5</v>
       </c>
       <c r="C9">
-        <v>5.6</v>
-      </c>
-      <c r="F9" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+        <v>4.66</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>6.5</v>
       </c>
@@ -1668,10 +1673,10 @@
         <v>6.5</v>
       </c>
       <c r="C10">
-        <v>6.3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+        <v>5.64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>7.5</v>
       </c>
@@ -1679,10 +1684,10 @@
         <v>7.5</v>
       </c>
       <c r="C11">
-        <v>6.7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+        <v>6.62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>8.5</v>
       </c>
@@ -1690,10 +1695,10 @@
         <v>8.5</v>
       </c>
       <c r="C12">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+        <v>7.59</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>9.5</v>
       </c>
@@ -1701,49 +1706,38 @@
         <v>9.5</v>
       </c>
       <c r="C13">
-        <v>7.6</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>10.5</v>
-      </c>
-      <c r="B14">
-        <v>10.5</v>
-      </c>
-      <c r="C14">
-        <v>8.4</v>
+        <v>8.5299999999999994</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B23" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" t="s">
         <v>11</v>
-      </c>
-      <c r="C23" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
@@ -1880,48 +1874,57 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>13</v>
-      </c>
-      <c r="B39" t="s">
-        <v>14</v>
-      </c>
-      <c r="C39" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B40">
-        <v>2</v>
-      </c>
-      <c r="C40">
-        <v>0.09</v>
+      <c r="A40" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>15</v>
-      </c>
-      <c r="B42">
-        <v>2.09</v>
-      </c>
-      <c r="C42">
-        <v>4.4999999999999998E-2</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
+        <v>17</v>
+      </c>
+      <c r="B42" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>12</v>
+      </c>
+      <c r="B43" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>14</v>
+      </c>
+      <c r="B45" t="s">
         <v>18</v>
       </c>
-      <c r="B44">
-        <v>1.57</v>
-      </c>
-      <c r="C44">
-        <v>1.4E-2</v>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>19</v>
+      </c>
+      <c r="B47" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>20</v>
+      </c>
+      <c r="B49" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>